<commit_message>
Close Universal Master at three and cut The Road Unrolls
Approves One More Dawn at 8 DP, The Mountain Walks and Touched by the Divine at 6 DP. Records CHG-UMA-001 through CHG-UMA-004.

The Universal ladder is now 13 Novice, 6 Adept and 3 Master. Book cards remain unchanged.
</commit_message>
<xml_diff>
--- a/review/abilities/workbooks/33_Master_Abilities.xlsx
+++ b/review/abilities/workbooks/33_Master_Abilities.xlsx
@@ -336,7 +336,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -783,7 +782,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The 87 shared Master (level 7) abilities. The 30 class signatures are excluded here and reviewed in the ten class workbooks.</t>
+          <t>The 87 shared Master (level 7) abilities plus the two new Universal Master abilities. The 30 class signatures are excluded here and reviewed in the ten class workbooks.</t>
         </is>
       </c>
     </row>
@@ -1149,8 +1148,8 @@
   </sheetData>
   <mergeCells count="23">
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A20:D20"/>
@@ -1193,7 +1192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V91"/>
+  <dimension ref="A1:V93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1230,7 +1229,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>87 shared cards. Signatures are excluded. Filter, decide, and add notes.</t>
+          <t>87 shared cards plus two new Universal Master cards. Signatures are excluded. Filter, decide, and add notes.</t>
         </is>
       </c>
     </row>
@@ -5257,8 +5256,16 @@
           <t>Re-tier to Novice 2 DP or add a Master-scale benefit and a discipline requirement.</t>
         </is>
       </c>
-      <c r="T41" s="7" t="inlineStr"/>
-      <c r="U41" s="7" t="inlineStr"/>
+      <c r="T41" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U41" s="7" t="inlineStr">
+        <is>
+          <t>Existing Universal Master; 8 DP confirmed 2026-10-29.</t>
+        </is>
+      </c>
       <c r="V41" s="7" t="inlineStr">
         <is>
           <t>one-more-dawn.md</t>
@@ -10536,6 +10543,231 @@
       <c r="V91" s="7" t="inlineStr">
         <is>
           <t>wear-the-great-beast.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>The Mountain Walks</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>the-mountain-walks</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Level 7</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Charge</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Main Action</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Brawn</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Self; one straight line up to your Speed.</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Instant.</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Once per scene; one line; uses your Main Action and movement for the turn.</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Charge in a straight line; push contacted creatures 2 squares with Stability; break barriers.</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>You must have movement remaining. Move in a straight line. When your line reaches a square occupied by a creature, push that creature 2 squares out of your path, applying Stability. If the creature leaves the square, you can continue through it. If the creature cannot leave, it is knocked Prone and your charge stops in the last legal square before it. Apply the normal collision rules.
+When your line reaches a nonmagical barrier no thicker than 1 square, the barrier breaks and leaves a passage. You can continue through the passage. The DA confirms the barrier is breakable and the line is clear enough for the charge.</t>
+        </is>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>MA1; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>the-mountain-walks.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Touched by the Divine</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>touched-by-the-divine</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Level 7</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Universal / Skill / Language / Passive</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>None (no roll)</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Self.</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Permanent.</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Purchase once.</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Understand every spoken language you hear.</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>You understand every spoken language you hear. Your own speech and literacy remain the languages you have learned.</t>
+        </is>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>MA2; approved 2026-10-29.</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>touched-by-the-divine.md</t>
         </is>
       </c>
     </row>
@@ -10704,8 +10936,16 @@
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>8 DP confirmed; premium Universal Master option; 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -11497,7 +11737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13566,7 +13806,7 @@
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>No requirement; policy gap (F02).</t>
+          <t>No requirement; Universal Master; 8 DP confirmed.</t>
         </is>
       </c>
     </row>
@@ -16249,6 +16489,110 @@
       <c r="K91" s="7" t="inlineStr">
         <is>
           <t>Single-discipline requirement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>The Mountain Walks</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>the-mountain-walks</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Main Action</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Movement</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Master.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Touched by the Divine</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>touched-by-the-divine</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Passive</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Utility</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>No requirement; Universal Master.</t>
         </is>
       </c>
     </row>
@@ -17168,80 +17512,336 @@
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1">
-      <c r="A5" s="7" t="inlineStr"/>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
-      <c r="K5" s="7" t="inlineStr"/>
-      <c r="L5" s="7" t="inlineStr"/>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" s="7" t="inlineStr"/>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UMA-001</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>UNI-04</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>one-more-dawn</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>One More Dawn</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>one-more-dawn.md</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Tier price</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Master 8 DP, no requirement, flagged High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Master 8 DP confirmed as the premium Universal option; purchase once; no requirement.</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>User confirmed 8 DP is warranted for One More Dawn.</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O5" s="7" t="inlineStr"/>
-      <c r="P5" s="7" t="inlineStr"/>
-      <c r="Q5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>Existing Universal Master; 8 DP confirmed.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="16.5" customHeight="1">
-      <c r="A6" s="9" t="inlineStr"/>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" s="9" t="inlineStr"/>
-      <c r="I6" s="9" t="inlineStr"/>
-      <c r="J6" s="9" t="inlineStr"/>
-      <c r="K6" s="9" t="inlineStr"/>
-      <c r="L6" s="9" t="inlineStr"/>
-      <c r="M6" s="9" t="inlineStr"/>
-      <c r="N6" s="9" t="inlineStr"/>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UMA-002</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>UNI-04</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>the-mountain-walks</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>The Mountain Walks</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>the-mountain-walks.md</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Main Action plus movement; straight-line charge; push contacted creatures 2 squares with Stability; break barriers; once per scene; 6 DP, Master, minimum level 7.</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
+        <is>
+          <t>Universal Master first pass; MA1 approved.</t>
+        </is>
+      </c>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O6" s="9" t="inlineStr"/>
-      <c r="P6" s="9" t="inlineStr"/>
-      <c r="Q6" s="9" t="inlineStr"/>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>MA1; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="16.5" customHeight="1">
-      <c r="A7" s="7" t="inlineStr"/>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr"/>
-      <c r="N7" s="7" t="inlineStr"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>CHG-UMA-003</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>UNI-04</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>touched-by-the-divine</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Touched by the Divine</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>touched-by-the-divine.md</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Passive; understand every spoken language you hear; permanent; 6 DP, Master, minimum level 7.</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>New ability</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Universal Master first pass; MA2 approved.</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O7" s="7" t="inlineStr"/>
-      <c r="P7" s="7" t="inlineStr"/>
-      <c r="Q7" s="7" t="inlineStr"/>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t>MA2; approved 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="16.5" customHeight="1">
-      <c r="A8" s="9" t="inlineStr"/>
-      <c r="B8" s="9" t="inlineStr"/>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="9" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-      <c r="L8" s="9" t="inlineStr"/>
-      <c r="M8" s="9" t="inlineStr"/>
-      <c r="N8" s="9" t="inlineStr"/>
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>CHG-UMA-004</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>UNI-04</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>the-road-unrolls</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>The Road Unrolls</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>the-road-unrolls.md</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Card proposal</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Proposed Master Universal at 6 DP</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Cut; the Master Universal set remains One More Dawn, The Mountain Walks and Touched by the Divine</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>User dropped the card to keep the set at three.</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Cut</t>
+        </is>
+      </c>
+      <c r="L8" s="9" t="inlineStr">
+        <is>
+          <t>Bruce</t>
+        </is>
+      </c>
+      <c r="M8" s="9" t="inlineStr">
+        <is>
+          <t>#1284</t>
+        </is>
+      </c>
+      <c r="N8" s="9" t="inlineStr">
+        <is>
+          <t>bruceamoser/heroes-of-legend-foundry#252</t>
+        </is>
+      </c>
       <c r="O8" s="9" t="inlineStr"/>
-      <c r="P8" s="9" t="inlineStr"/>
-      <c r="Q8" s="9" t="inlineStr"/>
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>MA3 cut 2026-10-29.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="16.5" customHeight="1">
       <c r="A9" s="7" t="inlineStr"/>

</xml_diff>